<commit_message>
Move the yearly flow point to Khajuriya ghat by the Pilibhit bypass
The ghat is at 28.3621 N, 79.4754 E, river km 29.4, not at Saidpur
Khajuria 4.6 km downstream. Its GEOGLOWS segment is 441105311
(km 27-29; contributing area about 148 km2, estimated), and MERIT-Hydro
puts 200 km2 of watershed above it. Flows, the yearly table, the
flow-history workbook, the watershed outline and the docs follow.
</commit_message>
<xml_diff>
--- a/data/nakatiya_yearly_observations.xlsx
+++ b/data/nakatiya_yearly_observations.xlsx
@@ -2678,22 +2678,22 @@
         <v>1940</v>
       </c>
       <c r="B41" t="n">
-        <v>0.408</v>
+        <v>0.34</v>
       </c>
       <c r="C41" t="n">
-        <v>1.094</v>
+        <v>0.912</v>
       </c>
       <c r="D41" t="n">
-        <v>0.091</v>
+        <v>0.075</v>
       </c>
       <c r="E41" t="n">
-        <v>0.244</v>
+        <v>0.2</v>
       </c>
       <c r="F41" t="n">
-        <v>0.285</v>
+        <v>0.255</v>
       </c>
       <c r="G41" t="n">
-        <v>0.738</v>
+        <v>0.661</v>
       </c>
       <c r="H41" t="n">
         <v>80.69</v>
@@ -2755,22 +2755,22 @@
         <v>1941</v>
       </c>
       <c r="B42" t="n">
-        <v>0.104</v>
+        <v>0.092</v>
       </c>
       <c r="C42" t="n">
-        <v>0.277</v>
+        <v>0.245</v>
       </c>
       <c r="D42" t="n">
-        <v>0.025</v>
+        <v>0.022</v>
       </c>
       <c r="E42" t="n">
-        <v>0.068</v>
+        <v>0.06</v>
       </c>
       <c r="F42" t="n">
-        <v>0.802</v>
+        <v>0.673</v>
       </c>
       <c r="G42" t="n">
-        <v>2.078</v>
+        <v>1.744</v>
       </c>
       <c r="H42" t="n">
         <v>149.59</v>
@@ -2832,10 +2832,10 @@
         <v>1942</v>
       </c>
       <c r="B43" t="n">
-        <v>0.305</v>
+        <v>0.28</v>
       </c>
       <c r="C43" t="n">
-        <v>0.8159999999999999</v>
+        <v>0.749</v>
       </c>
       <c r="D43" t="n">
         <v>0.007</v>
@@ -2844,10 +2844,10 @@
         <v>0.019</v>
       </c>
       <c r="F43" t="n">
-        <v>14.562</v>
+        <v>12.565</v>
       </c>
       <c r="G43" t="n">
-        <v>37.746</v>
+        <v>32.569</v>
       </c>
       <c r="H43" t="n">
         <v>171.58</v>
@@ -2909,22 +2909,22 @@
         <v>1943</v>
       </c>
       <c r="B44" t="n">
-        <v>0.63</v>
+        <v>0.492</v>
       </c>
       <c r="C44" t="n">
-        <v>1.688</v>
+        <v>1.318</v>
       </c>
       <c r="D44" t="n">
-        <v>0.097</v>
+        <v>0.077</v>
       </c>
       <c r="E44" t="n">
-        <v>0.26</v>
+        <v>0.206</v>
       </c>
       <c r="F44" t="n">
-        <v>21.87</v>
+        <v>17.839</v>
       </c>
       <c r="G44" t="n">
-        <v>56.687</v>
+        <v>46.24</v>
       </c>
       <c r="H44" t="n">
         <v>162.95</v>
@@ -2986,22 +2986,22 @@
         <v>1944</v>
       </c>
       <c r="B45" t="n">
-        <v>0.645</v>
+        <v>0.506</v>
       </c>
       <c r="C45" t="n">
-        <v>1.729</v>
+        <v>1.356</v>
       </c>
       <c r="D45" t="n">
-        <v>0.098</v>
+        <v>0.076</v>
       </c>
       <c r="E45" t="n">
-        <v>0.263</v>
+        <v>0.205</v>
       </c>
       <c r="F45" t="n">
-        <v>4.225</v>
+        <v>3.768</v>
       </c>
       <c r="G45" t="n">
-        <v>10.95</v>
+        <v>9.766999999999999</v>
       </c>
       <c r="H45" t="n">
         <v>173.82</v>
@@ -3063,22 +3063,22 @@
         <v>1945</v>
       </c>
       <c r="B46" t="n">
-        <v>0.301</v>
+        <v>0.245</v>
       </c>
       <c r="C46" t="n">
-        <v>0.8070000000000001</v>
+        <v>0.655</v>
       </c>
       <c r="D46" t="n">
-        <v>0.046</v>
+        <v>0.038</v>
       </c>
       <c r="E46" t="n">
-        <v>0.124</v>
+        <v>0.101</v>
       </c>
       <c r="F46" t="n">
-        <v>6.687</v>
+        <v>5.854</v>
       </c>
       <c r="G46" t="n">
-        <v>17.334</v>
+        <v>15.173</v>
       </c>
       <c r="H46" t="n">
         <v>38.96</v>
@@ -3140,22 +3140,22 @@
         <v>1946</v>
       </c>
       <c r="B47" t="n">
-        <v>0.575</v>
+        <v>0.471</v>
       </c>
       <c r="C47" t="n">
-        <v>1.54</v>
+        <v>1.262</v>
       </c>
       <c r="D47" t="n">
-        <v>0.077</v>
+        <v>0.063</v>
       </c>
       <c r="E47" t="n">
-        <v>0.206</v>
+        <v>0.169</v>
       </c>
       <c r="F47" t="n">
-        <v>1.514</v>
+        <v>1.269</v>
       </c>
       <c r="G47" t="n">
-        <v>3.924</v>
+        <v>3.29</v>
       </c>
       <c r="H47" t="n">
         <v>185.11</v>
@@ -3217,22 +3217,22 @@
         <v>1947</v>
       </c>
       <c r="B48" t="n">
-        <v>0.306</v>
+        <v>0.246</v>
       </c>
       <c r="C48" t="n">
-        <v>0.821</v>
+        <v>0.659</v>
       </c>
       <c r="D48" t="n">
-        <v>0.049</v>
+        <v>0.04</v>
       </c>
       <c r="E48" t="n">
-        <v>0.132</v>
+        <v>0.107</v>
       </c>
       <c r="F48" t="n">
-        <v>8.286</v>
+        <v>7.37</v>
       </c>
       <c r="G48" t="n">
-        <v>21.476</v>
+        <v>19.102</v>
       </c>
       <c r="H48" t="n">
         <v>123.85</v>
@@ -3294,22 +3294,22 @@
         <v>1948</v>
       </c>
       <c r="B49" t="n">
-        <v>0.607</v>
+        <v>0.482</v>
       </c>
       <c r="C49" t="n">
-        <v>1.626</v>
+        <v>1.291</v>
       </c>
       <c r="D49" t="n">
-        <v>0.08</v>
+        <v>0.065</v>
       </c>
       <c r="E49" t="n">
-        <v>0.214</v>
+        <v>0.174</v>
       </c>
       <c r="F49" t="n">
-        <v>9.851000000000001</v>
+        <v>8.564</v>
       </c>
       <c r="G49" t="n">
-        <v>25.535</v>
+        <v>22.197</v>
       </c>
       <c r="H49" t="n">
         <v>6.2</v>
@@ -3371,22 +3371,22 @@
         <v>1949</v>
       </c>
       <c r="B50" t="n">
-        <v>0.538</v>
+        <v>0.429</v>
       </c>
       <c r="C50" t="n">
-        <v>1.442</v>
+        <v>1.148</v>
       </c>
       <c r="D50" t="n">
-        <v>0.288</v>
+        <v>0.233</v>
       </c>
       <c r="E50" t="n">
-        <v>0.772</v>
+        <v>0.623</v>
       </c>
       <c r="F50" t="n">
-        <v>8.954000000000001</v>
+        <v>7.546</v>
       </c>
       <c r="G50" t="n">
-        <v>23.208</v>
+        <v>19.559</v>
       </c>
       <c r="H50" t="n">
         <v>30.83</v>
@@ -3448,22 +3448,22 @@
         <v>1950</v>
       </c>
       <c r="B51" t="n">
-        <v>0.675</v>
+        <v>0.532</v>
       </c>
       <c r="C51" t="n">
-        <v>1.807</v>
+        <v>1.425</v>
       </c>
       <c r="D51" t="n">
-        <v>0.122</v>
+        <v>0.096</v>
       </c>
       <c r="E51" t="n">
-        <v>0.327</v>
+        <v>0.258</v>
       </c>
       <c r="F51" t="n">
-        <v>5.257</v>
+        <v>4.683</v>
       </c>
       <c r="G51" t="n">
-        <v>13.625</v>
+        <v>12.139</v>
       </c>
       <c r="H51" t="n">
         <v>208.7</v>
@@ -3525,22 +3525,22 @@
         <v>1951</v>
       </c>
       <c r="B52" t="n">
-        <v>5.545</v>
+        <v>4.574</v>
       </c>
       <c r="C52" t="n">
-        <v>14.85</v>
+        <v>12.252</v>
       </c>
       <c r="D52" t="n">
-        <v>0.616</v>
+        <v>0.498</v>
       </c>
       <c r="E52" t="n">
-        <v>1.651</v>
+        <v>1.334</v>
       </c>
       <c r="F52" t="n">
-        <v>1.427</v>
+        <v>1.237</v>
       </c>
       <c r="G52" t="n">
-        <v>3.7</v>
+        <v>3.207</v>
       </c>
       <c r="H52" t="n">
         <v>24.81</v>
@@ -3602,22 +3602,22 @@
         <v>1952</v>
       </c>
       <c r="B53" t="n">
-        <v>0.891</v>
+        <v>0.738</v>
       </c>
       <c r="C53" t="n">
-        <v>2.386</v>
+        <v>1.978</v>
       </c>
       <c r="D53" t="n">
-        <v>0.524</v>
+        <v>0.46</v>
       </c>
       <c r="E53" t="n">
-        <v>1.403</v>
+        <v>1.231</v>
       </c>
       <c r="F53" t="n">
-        <v>6.534</v>
+        <v>5.375</v>
       </c>
       <c r="G53" t="n">
-        <v>16.936</v>
+        <v>13.931</v>
       </c>
       <c r="H53" t="n">
         <v>164.4</v>
@@ -3679,22 +3679,22 @@
         <v>1953</v>
       </c>
       <c r="B54" t="n">
-        <v>1.403</v>
+        <v>1.175</v>
       </c>
       <c r="C54" t="n">
-        <v>3.757</v>
+        <v>3.148</v>
       </c>
       <c r="D54" t="n">
-        <v>0.198</v>
+        <v>0.162</v>
       </c>
       <c r="E54" t="n">
-        <v>0.53</v>
+        <v>0.434</v>
       </c>
       <c r="F54" t="n">
-        <v>7.049</v>
+        <v>5.512</v>
       </c>
       <c r="G54" t="n">
-        <v>18.271</v>
+        <v>14.288</v>
       </c>
       <c r="H54" t="n">
         <v>93.51000000000001</v>
@@ -3756,22 +3756,22 @@
         <v>1954</v>
       </c>
       <c r="B55" t="n">
-        <v>0.856</v>
+        <v>0.704</v>
       </c>
       <c r="C55" t="n">
-        <v>2.292</v>
+        <v>1.885</v>
       </c>
       <c r="D55" t="n">
-        <v>0.163</v>
+        <v>0.134</v>
       </c>
       <c r="E55" t="n">
-        <v>0.436</v>
+        <v>0.359</v>
       </c>
       <c r="F55" t="n">
-        <v>6.536</v>
+        <v>5.173</v>
       </c>
       <c r="G55" t="n">
-        <v>16.941</v>
+        <v>13.408</v>
       </c>
       <c r="H55" t="n">
         <v>87.55</v>
@@ -3833,22 +3833,22 @@
         <v>1955</v>
       </c>
       <c r="B56" t="n">
-        <v>0.678</v>
+        <v>0.529</v>
       </c>
       <c r="C56" t="n">
-        <v>1.815</v>
+        <v>1.418</v>
       </c>
       <c r="D56" t="n">
-        <v>0.093</v>
+        <v>0.073</v>
       </c>
       <c r="E56" t="n">
-        <v>0.248</v>
+        <v>0.194</v>
       </c>
       <c r="F56" t="n">
-        <v>8.753</v>
+        <v>7.427</v>
       </c>
       <c r="G56" t="n">
-        <v>22.689</v>
+        <v>19.252</v>
       </c>
       <c r="H56" t="n">
         <v>182.75</v>
@@ -3910,22 +3910,22 @@
         <v>1956</v>
       </c>
       <c r="B57" t="n">
-        <v>0.92</v>
+        <v>0.726</v>
       </c>
       <c r="C57" t="n">
-        <v>2.463</v>
+        <v>1.945</v>
       </c>
       <c r="D57" t="n">
-        <v>0.105</v>
+        <v>0.082</v>
       </c>
       <c r="E57" t="n">
-        <v>0.281</v>
+        <v>0.219</v>
       </c>
       <c r="F57" t="n">
-        <v>6.925</v>
+        <v>5.765</v>
       </c>
       <c r="G57" t="n">
-        <v>17.949</v>
+        <v>14.943</v>
       </c>
       <c r="H57" t="n">
         <v>130.89</v>
@@ -3987,22 +3987,22 @@
         <v>1957</v>
       </c>
       <c r="B58" t="n">
-        <v>0.979</v>
+        <v>0.782</v>
       </c>
       <c r="C58" t="n">
-        <v>2.623</v>
+        <v>2.095</v>
       </c>
       <c r="D58" t="n">
-        <v>0.118</v>
+        <v>0.094</v>
       </c>
       <c r="E58" t="n">
-        <v>0.316</v>
+        <v>0.251</v>
       </c>
       <c r="F58" t="n">
-        <v>29.503</v>
+        <v>23.484</v>
       </c>
       <c r="G58" t="n">
-        <v>76.471</v>
+        <v>60.87</v>
       </c>
       <c r="H58" t="n">
         <v>82.89</v>
@@ -4064,22 +4064,22 @@
         <v>1958</v>
       </c>
       <c r="B59" t="n">
-        <v>0.637</v>
+        <v>0.501</v>
       </c>
       <c r="C59" t="n">
-        <v>1.706</v>
+        <v>1.341</v>
       </c>
       <c r="D59" t="n">
-        <v>0.112</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="E59" t="n">
-        <v>0.3</v>
+        <v>0.233</v>
       </c>
       <c r="F59" t="n">
-        <v>14.833</v>
+        <v>12.204</v>
       </c>
       <c r="G59" t="n">
-        <v>38.447</v>
+        <v>31.632</v>
       </c>
       <c r="H59" t="n">
         <v>165.57</v>
@@ -4141,22 +4141,22 @@
         <v>1959</v>
       </c>
       <c r="B60" t="n">
-        <v>0.871</v>
+        <v>0.6870000000000001</v>
       </c>
       <c r="C60" t="n">
-        <v>2.333</v>
+        <v>1.841</v>
       </c>
       <c r="D60" t="n">
-        <v>0.205</v>
+        <v>0.163</v>
       </c>
       <c r="E60" t="n">
-        <v>0.55</v>
+        <v>0.435</v>
       </c>
       <c r="F60" t="n">
-        <v>6.388</v>
+        <v>5.629</v>
       </c>
       <c r="G60" t="n">
-        <v>16.559</v>
+        <v>14.59</v>
       </c>
       <c r="H60" t="n">
         <v>44.63</v>
@@ -4218,22 +4218,22 @@
         <v>1960</v>
       </c>
       <c r="B61" t="n">
-        <v>0.929</v>
+        <v>0.729</v>
       </c>
       <c r="C61" t="n">
-        <v>2.489</v>
+        <v>1.953</v>
       </c>
       <c r="D61" t="n">
-        <v>0.131</v>
+        <v>0.103</v>
       </c>
       <c r="E61" t="n">
-        <v>0.351</v>
+        <v>0.276</v>
       </c>
       <c r="F61" t="n">
-        <v>11.14</v>
+        <v>9.25</v>
       </c>
       <c r="G61" t="n">
-        <v>28.875</v>
+        <v>23.976</v>
       </c>
       <c r="H61" t="n">
         <v>124.37</v>
@@ -4295,22 +4295,22 @@
         <v>1961</v>
       </c>
       <c r="B62" t="n">
-        <v>1.093</v>
+        <v>0.873</v>
       </c>
       <c r="C62" t="n">
-        <v>2.926</v>
+        <v>2.337</v>
       </c>
       <c r="D62" t="n">
-        <v>0.294</v>
+        <v>0.237</v>
       </c>
       <c r="E62" t="n">
-        <v>0.786</v>
+        <v>0.636</v>
       </c>
       <c r="F62" t="n">
-        <v>13.069</v>
+        <v>11.082</v>
       </c>
       <c r="G62" t="n">
-        <v>33.874</v>
+        <v>28.725</v>
       </c>
       <c r="H62" t="n">
         <v>186.24</v>
@@ -4372,22 +4372,22 @@
         <v>1962</v>
       </c>
       <c r="B63" t="n">
-        <v>1.173</v>
+        <v>0.945</v>
       </c>
       <c r="C63" t="n">
-        <v>3.142</v>
+        <v>2.531</v>
       </c>
       <c r="D63" t="n">
-        <v>0.218</v>
+        <v>0.177</v>
       </c>
       <c r="E63" t="n">
-        <v>0.585</v>
+        <v>0.473</v>
       </c>
       <c r="F63" t="n">
-        <v>27.54</v>
+        <v>22.74</v>
       </c>
       <c r="G63" t="n">
-        <v>71.384</v>
+        <v>58.941</v>
       </c>
       <c r="H63" t="n">
         <v>116.62</v>
@@ -4449,22 +4449,22 @@
         <v>1963</v>
       </c>
       <c r="B64" t="n">
-        <v>0.789</v>
+        <v>0.624</v>
       </c>
       <c r="C64" t="n">
-        <v>2.114</v>
+        <v>1.672</v>
       </c>
       <c r="D64" t="n">
-        <v>0.109</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="E64" t="n">
-        <v>0.292</v>
+        <v>0.224</v>
       </c>
       <c r="F64" t="n">
-        <v>22.261</v>
+        <v>18.327</v>
       </c>
       <c r="G64" t="n">
-        <v>57.7</v>
+        <v>47.504</v>
       </c>
       <c r="H64" t="n">
         <v>128.78</v>
@@ -4526,22 +4526,22 @@
         <v>1964</v>
       </c>
       <c r="B65" t="n">
-        <v>0.449</v>
+        <v>0.352</v>
       </c>
       <c r="C65" t="n">
-        <v>1.203</v>
+        <v>0.9419999999999999</v>
       </c>
       <c r="D65" t="n">
-        <v>0.08799999999999999</v>
+        <v>0.07000000000000001</v>
       </c>
       <c r="E65" t="n">
-        <v>0.235</v>
+        <v>0.187</v>
       </c>
       <c r="F65" t="n">
-        <v>41.765</v>
+        <v>34.449</v>
       </c>
       <c r="G65" t="n">
-        <v>108.255</v>
+        <v>89.291</v>
       </c>
       <c r="H65" t="n">
         <v>92.36</v>
@@ -4603,22 +4603,22 @@
         <v>1965</v>
       </c>
       <c r="B66" t="n">
-        <v>0.5659999999999999</v>
+        <v>0.444</v>
       </c>
       <c r="C66" t="n">
-        <v>1.516</v>
+        <v>1.189</v>
       </c>
       <c r="D66" t="n">
-        <v>0.112</v>
+        <v>0.08699999999999999</v>
       </c>
       <c r="E66" t="n">
-        <v>0.299</v>
+        <v>0.233</v>
       </c>
       <c r="F66" t="n">
-        <v>0.9370000000000001</v>
+        <v>0.764</v>
       </c>
       <c r="G66" t="n">
-        <v>2.43</v>
+        <v>1.979</v>
       </c>
       <c r="H66" t="n">
         <v>15.15</v>
@@ -4680,22 +4680,22 @@
         <v>1966</v>
       </c>
       <c r="B67" t="n">
-        <v>0.217</v>
+        <v>0.177</v>
       </c>
       <c r="C67" t="n">
-        <v>0.581</v>
+        <v>0.473</v>
       </c>
       <c r="D67" t="n">
-        <v>0.05</v>
+        <v>0.04</v>
       </c>
       <c r="E67" t="n">
-        <v>0.135</v>
+        <v>0.108</v>
       </c>
       <c r="F67" t="n">
-        <v>3.085</v>
+        <v>2.594</v>
       </c>
       <c r="G67" t="n">
-        <v>7.996</v>
+        <v>6.725</v>
       </c>
       <c r="H67" t="n">
         <v>127.76</v>
@@ -4757,22 +4757,22 @@
         <v>1967</v>
       </c>
       <c r="B68" t="n">
-        <v>0.373</v>
+        <v>0.297</v>
       </c>
       <c r="C68" t="n">
-        <v>0.998</v>
+        <v>0.795</v>
       </c>
       <c r="D68" t="n">
-        <v>0.103</v>
+        <v>0.081</v>
       </c>
       <c r="E68" t="n">
-        <v>0.276</v>
+        <v>0.216</v>
       </c>
       <c r="F68" t="n">
-        <v>14.586</v>
+        <v>11.504</v>
       </c>
       <c r="G68" t="n">
-        <v>37.806</v>
+        <v>29.818</v>
       </c>
       <c r="H68" t="n">
         <v>174.04</v>
@@ -4834,22 +4834,22 @@
         <v>1968</v>
       </c>
       <c r="B69" t="n">
-        <v>0.784</v>
+        <v>0.618</v>
       </c>
       <c r="C69" t="n">
-        <v>2.099</v>
+        <v>1.656</v>
       </c>
       <c r="D69" t="n">
-        <v>0.167</v>
+        <v>0.132</v>
       </c>
       <c r="E69" t="n">
-        <v>0.448</v>
+        <v>0.354</v>
       </c>
       <c r="F69" t="n">
-        <v>8.561</v>
+        <v>7.094</v>
       </c>
       <c r="G69" t="n">
-        <v>22.189</v>
+        <v>18.389</v>
       </c>
       <c r="H69" t="n">
         <v>208.83</v>
@@ -4911,22 +4911,22 @@
         <v>1969</v>
       </c>
       <c r="B70" t="n">
-        <v>0.677</v>
+        <v>0.543</v>
       </c>
       <c r="C70" t="n">
-        <v>1.814</v>
+        <v>1.455</v>
       </c>
       <c r="D70" t="n">
-        <v>0.171</v>
+        <v>0.141</v>
       </c>
       <c r="E70" t="n">
-        <v>0.459</v>
+        <v>0.378</v>
       </c>
       <c r="F70" t="n">
-        <v>11.619</v>
+        <v>9.372</v>
       </c>
       <c r="G70" t="n">
-        <v>30.117</v>
+        <v>24.291</v>
       </c>
       <c r="H70" t="n">
         <v>20.56</v>
@@ -4988,22 +4988,22 @@
         <v>1970</v>
       </c>
       <c r="B71" t="n">
-        <v>1.046</v>
+        <v>0.8</v>
       </c>
       <c r="C71" t="n">
-        <v>2.802</v>
+        <v>2.142</v>
       </c>
       <c r="D71" t="n">
-        <v>0.195</v>
+        <v>0.156</v>
       </c>
       <c r="E71" t="n">
-        <v>0.524</v>
+        <v>0.417</v>
       </c>
       <c r="F71" t="n">
-        <v>3.585</v>
+        <v>3.231</v>
       </c>
       <c r="G71" t="n">
-        <v>9.292</v>
+        <v>8.375999999999999</v>
       </c>
       <c r="H71" t="n">
         <v>182.65</v>
@@ -5065,22 +5065,22 @@
         <v>1971</v>
       </c>
       <c r="B72" t="n">
-        <v>0.709</v>
+        <v>0.604</v>
       </c>
       <c r="C72" t="n">
-        <v>1.898</v>
+        <v>1.617</v>
       </c>
       <c r="D72" t="n">
-        <v>0.221</v>
+        <v>0.183</v>
       </c>
       <c r="E72" t="n">
-        <v>0.593</v>
+        <v>0.489</v>
       </c>
       <c r="F72" t="n">
-        <v>24.867</v>
+        <v>20.362</v>
       </c>
       <c r="G72" t="n">
-        <v>64.45399999999999</v>
+        <v>52.777</v>
       </c>
       <c r="H72" t="n">
         <v>156.27</v>
@@ -5142,22 +5142,22 @@
         <v>1972</v>
       </c>
       <c r="B73" t="n">
-        <v>0.754</v>
+        <v>0.605</v>
       </c>
       <c r="C73" t="n">
-        <v>2.018</v>
+        <v>1.622</v>
       </c>
       <c r="D73" t="n">
-        <v>0.175</v>
+        <v>0.14</v>
       </c>
       <c r="E73" t="n">
-        <v>0.468</v>
+        <v>0.374</v>
       </c>
       <c r="F73" t="n">
-        <v>11.399</v>
+        <v>9.507</v>
       </c>
       <c r="G73" t="n">
-        <v>29.545</v>
+        <v>24.643</v>
       </c>
       <c r="H73" t="n">
         <v>41.38</v>
@@ -5219,22 +5219,22 @@
         <v>1973</v>
       </c>
       <c r="B74" t="n">
-        <v>0.536</v>
+        <v>0.454</v>
       </c>
       <c r="C74" t="n">
-        <v>1.435</v>
+        <v>1.217</v>
       </c>
       <c r="D74" t="n">
-        <v>0.119</v>
+        <v>0.1</v>
       </c>
       <c r="E74" t="n">
-        <v>0.319</v>
+        <v>0.267</v>
       </c>
       <c r="F74" t="n">
-        <v>8.696</v>
+        <v>7.106</v>
       </c>
       <c r="G74" t="n">
-        <v>22.54</v>
+        <v>18.419</v>
       </c>
       <c r="H74" t="n">
         <v>332.14</v>
@@ -5296,22 +5296,22 @@
         <v>1974</v>
       </c>
       <c r="B75" t="n">
-        <v>0.958</v>
+        <v>0.752</v>
       </c>
       <c r="C75" t="n">
-        <v>2.567</v>
+        <v>2.013</v>
       </c>
       <c r="D75" t="n">
-        <v>0.149</v>
+        <v>0.114</v>
       </c>
       <c r="E75" t="n">
-        <v>0.399</v>
+        <v>0.306</v>
       </c>
       <c r="F75" t="n">
-        <v>2.046</v>
+        <v>1.694</v>
       </c>
       <c r="G75" t="n">
-        <v>5.304</v>
+        <v>4.391</v>
       </c>
       <c r="H75" t="n">
         <v>69.69</v>
@@ -5373,22 +5373,22 @@
         <v>1975</v>
       </c>
       <c r="B76" t="n">
-        <v>0.379</v>
+        <v>0.3</v>
       </c>
       <c r="C76" t="n">
-        <v>1.016</v>
+        <v>0.804</v>
       </c>
       <c r="D76" t="n">
-        <v>0.08699999999999999</v>
+        <v>0.066</v>
       </c>
       <c r="E76" t="n">
-        <v>0.233</v>
+        <v>0.178</v>
       </c>
       <c r="F76" t="n">
-        <v>16.155</v>
+        <v>13.433</v>
       </c>
       <c r="G76" t="n">
-        <v>41.874</v>
+        <v>34.817</v>
       </c>
       <c r="H76" t="n">
         <v>371.58</v>
@@ -5450,22 +5450,22 @@
         <v>1976</v>
       </c>
       <c r="B77" t="n">
-        <v>0.643</v>
+        <v>0.507</v>
       </c>
       <c r="C77" t="n">
-        <v>1.722</v>
+        <v>1.358</v>
       </c>
       <c r="D77" t="n">
-        <v>0.137</v>
+        <v>0.108</v>
       </c>
       <c r="E77" t="n">
-        <v>0.368</v>
+        <v>0.289</v>
       </c>
       <c r="F77" t="n">
-        <v>9.956</v>
+        <v>8.353</v>
       </c>
       <c r="G77" t="n">
-        <v>25.806</v>
+        <v>21.651</v>
       </c>
       <c r="H77" t="n">
         <v>100.91</v>
@@ -5527,22 +5527,22 @@
         <v>1977</v>
       </c>
       <c r="B78" t="n">
-        <v>0.627</v>
+        <v>0.499</v>
       </c>
       <c r="C78" t="n">
-        <v>1.679</v>
+        <v>1.336</v>
       </c>
       <c r="D78" t="n">
-        <v>0.161</v>
+        <v>0.128</v>
       </c>
       <c r="E78" t="n">
-        <v>0.431</v>
+        <v>0.344</v>
       </c>
       <c r="F78" t="n">
-        <v>6.708</v>
+        <v>5.975</v>
       </c>
       <c r="G78" t="n">
-        <v>17.386</v>
+        <v>15.488</v>
       </c>
       <c r="H78" t="n">
         <v>61.46</v>
@@ -5604,22 +5604,22 @@
         <v>1978</v>
       </c>
       <c r="B79" t="n">
-        <v>0.659</v>
+        <v>0.539</v>
       </c>
       <c r="C79" t="n">
-        <v>1.764</v>
+        <v>1.444</v>
       </c>
       <c r="D79" t="n">
-        <v>0.15</v>
+        <v>0.124</v>
       </c>
       <c r="E79" t="n">
-        <v>0.403</v>
+        <v>0.331</v>
       </c>
       <c r="F79" t="n">
-        <v>6.017</v>
+        <v>4.848</v>
       </c>
       <c r="G79" t="n">
-        <v>15.596</v>
+        <v>12.566</v>
       </c>
       <c r="H79" t="n">
         <v>374.47</v>
@@ -5681,22 +5681,22 @@
         <v>1979</v>
       </c>
       <c r="B80" t="n">
-        <v>0.575</v>
+        <v>0.467</v>
       </c>
       <c r="C80" t="n">
-        <v>1.539</v>
+        <v>1.252</v>
       </c>
       <c r="D80" t="n">
-        <v>0.405</v>
+        <v>0.354</v>
       </c>
       <c r="E80" t="n">
-        <v>1.083</v>
+        <v>0.947</v>
       </c>
       <c r="F80" t="n">
-        <v>0.246</v>
+        <v>0.225</v>
       </c>
       <c r="G80" t="n">
-        <v>0.637</v>
+        <v>0.584</v>
       </c>
       <c r="H80" t="n">
         <v>109.56</v>
@@ -5758,22 +5758,22 @@
         <v>1980</v>
       </c>
       <c r="B81" t="n">
-        <v>0.095</v>
+        <v>0.08500000000000001</v>
       </c>
       <c r="C81" t="n">
-        <v>0.256</v>
+        <v>0.229</v>
       </c>
       <c r="D81" t="n">
-        <v>0.035</v>
+        <v>0.031</v>
       </c>
       <c r="E81" t="n">
-        <v>0.093</v>
+        <v>0.083</v>
       </c>
       <c r="F81" t="n">
-        <v>4.097</v>
+        <v>3.136</v>
       </c>
       <c r="G81" t="n">
-        <v>10.62</v>
+        <v>8.129</v>
       </c>
       <c r="H81" t="n">
         <v>95.56999999999999</v>
@@ -5835,22 +5835,22 @@
         <v>1981</v>
       </c>
       <c r="B82" t="n">
-        <v>0.6</v>
+        <v>0.48</v>
       </c>
       <c r="C82" t="n">
-        <v>1.607</v>
+        <v>1.286</v>
       </c>
       <c r="D82" t="n">
-        <v>0.178</v>
+        <v>0.143</v>
       </c>
       <c r="E82" t="n">
-        <v>0.478</v>
+        <v>0.384</v>
       </c>
       <c r="F82" t="n">
-        <v>3.129</v>
+        <v>2.633</v>
       </c>
       <c r="G82" t="n">
-        <v>8.109999999999999</v>
+        <v>6.825</v>
       </c>
       <c r="H82" t="n">
         <v>138.96</v>
@@ -5912,22 +5912,22 @@
         <v>1982</v>
       </c>
       <c r="B83" t="n">
-        <v>0.477</v>
+        <v>0.395</v>
       </c>
       <c r="C83" t="n">
-        <v>1.279</v>
+        <v>1.057</v>
       </c>
       <c r="D83" t="n">
-        <v>0.231</v>
+        <v>0.19</v>
       </c>
       <c r="E83" t="n">
-        <v>0.619</v>
+        <v>0.508</v>
       </c>
       <c r="F83" t="n">
-        <v>6.131</v>
+        <v>4.983</v>
       </c>
       <c r="G83" t="n">
-        <v>15.891</v>
+        <v>12.915</v>
       </c>
       <c r="H83" t="n">
         <v>90.89</v>
@@ -5989,22 +5989,22 @@
         <v>1983</v>
       </c>
       <c r="B84" t="n">
-        <v>0.545</v>
+        <v>0.457</v>
       </c>
       <c r="C84" t="n">
-        <v>1.46</v>
+        <v>1.225</v>
       </c>
       <c r="D84" t="n">
-        <v>0.165</v>
+        <v>0.136</v>
       </c>
       <c r="E84" t="n">
-        <v>0.443</v>
+        <v>0.364</v>
       </c>
       <c r="F84" t="n">
-        <v>19.805</v>
+        <v>15.624</v>
       </c>
       <c r="G84" t="n">
-        <v>51.335</v>
+        <v>40.497</v>
       </c>
       <c r="H84" t="n">
         <v>146.77</v>
@@ -6066,22 +6066,22 @@
         <v>1984</v>
       </c>
       <c r="B85" t="n">
-        <v>0.728</v>
+        <v>0.57</v>
       </c>
       <c r="C85" t="n">
-        <v>1.95</v>
+        <v>1.526</v>
       </c>
       <c r="D85" t="n">
-        <v>0.142</v>
+        <v>0.111</v>
       </c>
       <c r="E85" t="n">
-        <v>0.379</v>
+        <v>0.296</v>
       </c>
       <c r="F85" t="n">
-        <v>3.865</v>
+        <v>3.155</v>
       </c>
       <c r="G85" t="n">
-        <v>10.018</v>
+        <v>8.177</v>
       </c>
       <c r="H85" t="n">
         <v>339.13</v>
@@ -6143,22 +6143,22 @@
         <v>1985</v>
       </c>
       <c r="B86" t="n">
-        <v>0.572</v>
+        <v>0.455</v>
       </c>
       <c r="C86" t="n">
-        <v>1.531</v>
+        <v>1.218</v>
       </c>
       <c r="D86" t="n">
-        <v>0.101</v>
+        <v>0.078</v>
       </c>
       <c r="E86" t="n">
-        <v>0.27</v>
+        <v>0.209</v>
       </c>
       <c r="F86" t="n">
-        <v>22.953</v>
+        <v>18.562</v>
       </c>
       <c r="G86" t="n">
-        <v>59.495</v>
+        <v>48.113</v>
       </c>
       <c r="H86" t="n">
         <v>96.37</v>
@@ -6224,22 +6224,22 @@
         <v>1986</v>
       </c>
       <c r="B87" t="n">
-        <v>1.117</v>
+        <v>0.89</v>
       </c>
       <c r="C87" t="n">
-        <v>2.993</v>
+        <v>2.384</v>
       </c>
       <c r="D87" t="n">
-        <v>0.382</v>
+        <v>0.319</v>
       </c>
       <c r="E87" t="n">
-        <v>1.024</v>
+        <v>0.854</v>
       </c>
       <c r="F87" t="n">
-        <v>0.8129999999999999</v>
+        <v>0.6820000000000001</v>
       </c>
       <c r="G87" t="n">
-        <v>2.108</v>
+        <v>1.767</v>
       </c>
       <c r="H87" t="n">
         <v>88.15000000000001</v>
@@ -6305,22 +6305,22 @@
         <v>1987</v>
       </c>
       <c r="B88" t="n">
-        <v>0.231</v>
+        <v>0.191</v>
       </c>
       <c r="C88" t="n">
-        <v>0.618</v>
+        <v>0.511</v>
       </c>
       <c r="D88" t="n">
-        <v>0.199</v>
+        <v>0.17</v>
       </c>
       <c r="E88" t="n">
-        <v>0.534</v>
+        <v>0.456</v>
       </c>
       <c r="F88" t="n">
-        <v>0.856</v>
+        <v>0.668</v>
       </c>
       <c r="G88" t="n">
-        <v>2.219</v>
+        <v>1.731</v>
       </c>
       <c r="H88" t="n">
         <v>64.09</v>
@@ -6386,22 +6386,22 @@
         <v>1988</v>
       </c>
       <c r="B89" t="n">
-        <v>0.014</v>
+        <v>0.012</v>
       </c>
       <c r="C89" t="n">
-        <v>0.038</v>
+        <v>0.032</v>
       </c>
       <c r="D89" t="n">
         <v>0.005</v>
       </c>
       <c r="E89" t="n">
-        <v>0.014</v>
+        <v>0.012</v>
       </c>
       <c r="F89" t="n">
-        <v>5.982</v>
+        <v>5.006</v>
       </c>
       <c r="G89" t="n">
-        <v>15.506</v>
+        <v>12.975</v>
       </c>
       <c r="H89" t="n">
         <v>84.54000000000001</v>
@@ -6467,22 +6467,22 @@
         <v>1989</v>
       </c>
       <c r="B90" t="n">
-        <v>0.617</v>
+        <v>0.499</v>
       </c>
       <c r="C90" t="n">
-        <v>1.653</v>
+        <v>1.337</v>
       </c>
       <c r="D90" t="n">
-        <v>0.126</v>
+        <v>0.102</v>
       </c>
       <c r="E90" t="n">
-        <v>0.339</v>
+        <v>0.272</v>
       </c>
       <c r="F90" t="n">
-        <v>2.711</v>
+        <v>2.252</v>
       </c>
       <c r="G90" t="n">
-        <v>7.027</v>
+        <v>5.838</v>
       </c>
       <c r="H90" t="n">
         <v>167.36</v>
@@ -6548,22 +6548,22 @@
         <v>1990</v>
       </c>
       <c r="B91" t="n">
-        <v>0.263</v>
+        <v>0.227</v>
       </c>
       <c r="C91" t="n">
-        <v>0.704</v>
+        <v>0.609</v>
       </c>
       <c r="D91" t="n">
-        <v>0.18</v>
+        <v>0.146</v>
       </c>
       <c r="E91" t="n">
-        <v>0.482</v>
+        <v>0.392</v>
       </c>
       <c r="F91" t="n">
-        <v>10.448</v>
+        <v>9.045</v>
       </c>
       <c r="G91" t="n">
-        <v>27.08</v>
+        <v>23.445</v>
       </c>
       <c r="H91" t="n">
         <v>104.63</v>
@@ -6629,22 +6629,22 @@
         <v>1991</v>
       </c>
       <c r="B92" t="n">
-        <v>0.799</v>
+        <v>0.644</v>
       </c>
       <c r="C92" t="n">
-        <v>2.139</v>
+        <v>1.725</v>
       </c>
       <c r="D92" t="n">
-        <v>0.135</v>
+        <v>0.107</v>
       </c>
       <c r="E92" t="n">
-        <v>0.361</v>
+        <v>0.286</v>
       </c>
       <c r="F92" t="n">
-        <v>4.135</v>
+        <v>3.461</v>
       </c>
       <c r="G92" t="n">
-        <v>10.719</v>
+        <v>8.971</v>
       </c>
       <c r="H92" t="n">
         <v>60.01</v>
@@ -6718,22 +6718,22 @@
         <v>1992</v>
       </c>
       <c r="B93" t="n">
-        <v>0.525</v>
+        <v>0.448</v>
       </c>
       <c r="C93" t="n">
-        <v>1.405</v>
+        <v>1.199</v>
       </c>
       <c r="D93" t="n">
-        <v>0.147</v>
+        <v>0.124</v>
       </c>
       <c r="E93" t="n">
-        <v>0.394</v>
+        <v>0.331</v>
       </c>
       <c r="F93" t="n">
-        <v>2.874</v>
+        <v>2.593</v>
       </c>
       <c r="G93" t="n">
-        <v>7.45</v>
+        <v>6.722</v>
       </c>
       <c r="H93" t="n">
         <v>436.35</v>
@@ -6811,22 +6811,22 @@
         <v>1993</v>
       </c>
       <c r="B94" t="n">
-        <v>0.634</v>
+        <v>0.541</v>
       </c>
       <c r="C94" t="n">
-        <v>1.697</v>
+        <v>1.449</v>
       </c>
       <c r="D94" t="n">
-        <v>0.149</v>
+        <v>0.125</v>
       </c>
       <c r="E94" t="n">
-        <v>0.4</v>
+        <v>0.335</v>
       </c>
       <c r="F94" t="n">
-        <v>22.086</v>
+        <v>19.73</v>
       </c>
       <c r="G94" t="n">
-        <v>57.246</v>
+        <v>51.141</v>
       </c>
       <c r="H94" t="n">
         <v>132.05</v>
@@ -6904,22 +6904,22 @@
         <v>1994</v>
       </c>
       <c r="B95" t="n">
-        <v>0.596</v>
+        <v>0.485</v>
       </c>
       <c r="C95" t="n">
-        <v>1.597</v>
+        <v>1.299</v>
       </c>
       <c r="D95" t="n">
-        <v>0.121</v>
+        <v>0.096</v>
       </c>
       <c r="E95" t="n">
-        <v>0.324</v>
+        <v>0.257</v>
       </c>
       <c r="F95" t="n">
-        <v>3.334</v>
+        <v>2.972</v>
       </c>
       <c r="G95" t="n">
-        <v>8.641</v>
+        <v>7.703</v>
       </c>
       <c r="H95" t="n">
         <v>102.67</v>
@@ -7013,22 +7013,22 @@
         <v>1995</v>
       </c>
       <c r="B96" t="n">
-        <v>0.666</v>
+        <v>0.545</v>
       </c>
       <c r="C96" t="n">
-        <v>1.784</v>
+        <v>1.459</v>
       </c>
       <c r="D96" t="n">
-        <v>0.121</v>
+        <v>0.099</v>
       </c>
       <c r="E96" t="n">
-        <v>0.325</v>
+        <v>0.264</v>
       </c>
       <c r="F96" t="n">
-        <v>6.897</v>
+        <v>6.005</v>
       </c>
       <c r="G96" t="n">
-        <v>17.877</v>
+        <v>15.564</v>
       </c>
       <c r="H96" t="n">
         <v>116.12</v>
@@ -7122,22 +7122,22 @@
         <v>1996</v>
       </c>
       <c r="B97" t="n">
-        <v>0.533</v>
+        <v>0.437</v>
       </c>
       <c r="C97" t="n">
-        <v>1.428</v>
+        <v>1.17</v>
       </c>
       <c r="D97" t="n">
-        <v>0.138</v>
+        <v>0.112</v>
       </c>
       <c r="E97" t="n">
-        <v>0.37</v>
+        <v>0.3</v>
       </c>
       <c r="F97" t="n">
-        <v>19.215</v>
+        <v>15.448</v>
       </c>
       <c r="G97" t="n">
-        <v>49.804</v>
+        <v>40.04</v>
       </c>
       <c r="H97" t="n">
         <v>151.27</v>
@@ -7231,22 +7231,22 @@
         <v>1997</v>
       </c>
       <c r="B98" t="n">
-        <v>0.665</v>
+        <v>0.524</v>
       </c>
       <c r="C98" t="n">
-        <v>1.782</v>
+        <v>1.402</v>
       </c>
       <c r="D98" t="n">
-        <v>0.173</v>
+        <v>0.137</v>
       </c>
       <c r="E98" t="n">
-        <v>0.464</v>
+        <v>0.367</v>
       </c>
       <c r="F98" t="n">
-        <v>2.378</v>
+        <v>1.99</v>
       </c>
       <c r="G98" t="n">
-        <v>6.164</v>
+        <v>5.157</v>
       </c>
       <c r="H98" t="n">
         <v>91.28</v>
@@ -7320,22 +7320,22 @@
         <v>1998</v>
       </c>
       <c r="B99" t="n">
-        <v>0.758</v>
+        <v>0.601</v>
       </c>
       <c r="C99" t="n">
-        <v>2.03</v>
+        <v>1.61</v>
       </c>
       <c r="D99" t="n">
-        <v>0.859</v>
+        <v>0.715</v>
       </c>
       <c r="E99" t="n">
-        <v>2.301</v>
+        <v>1.915</v>
       </c>
       <c r="F99" t="n">
-        <v>6.411</v>
+        <v>5.203</v>
       </c>
       <c r="G99" t="n">
-        <v>16.618</v>
+        <v>13.485</v>
       </c>
       <c r="H99" t="n">
         <v>110.34</v>
@@ -7429,22 +7429,22 @@
         <v>1999</v>
       </c>
       <c r="B100" t="n">
-        <v>1.015</v>
+        <v>0.8090000000000001</v>
       </c>
       <c r="C100" t="n">
-        <v>2.717</v>
+        <v>2.168</v>
       </c>
       <c r="D100" t="n">
-        <v>0.19</v>
+        <v>0.151</v>
       </c>
       <c r="E100" t="n">
-        <v>0.509</v>
+        <v>0.403</v>
       </c>
       <c r="F100" t="n">
-        <v>4.217</v>
+        <v>3.741</v>
       </c>
       <c r="G100" t="n">
-        <v>10.931</v>
+        <v>9.698</v>
       </c>
       <c r="H100" t="n">
         <v>77.84999999999999</v>
@@ -7538,22 +7538,22 @@
         <v>2000</v>
       </c>
       <c r="B101" t="n">
-        <v>0.595</v>
+        <v>0.516</v>
       </c>
       <c r="C101" t="n">
-        <v>1.593</v>
+        <v>1.382</v>
       </c>
       <c r="D101" t="n">
-        <v>0.164</v>
+        <v>0.139</v>
       </c>
       <c r="E101" t="n">
-        <v>0.44</v>
+        <v>0.373</v>
       </c>
       <c r="F101" t="n">
-        <v>4.813</v>
+        <v>4.218</v>
       </c>
       <c r="G101" t="n">
-        <v>12.476</v>
+        <v>10.934</v>
       </c>
       <c r="H101" t="n">
         <v>292.48</v>
@@ -7647,22 +7647,22 @@
         <v>2001</v>
       </c>
       <c r="B102" t="n">
-        <v>0.776</v>
+        <v>0.62</v>
       </c>
       <c r="C102" t="n">
-        <v>2.078</v>
+        <v>1.661</v>
       </c>
       <c r="D102" t="n">
-        <v>0.217</v>
+        <v>0.173</v>
       </c>
       <c r="E102" t="n">
-        <v>0.581</v>
+        <v>0.464</v>
       </c>
       <c r="F102" t="n">
-        <v>1.12</v>
+        <v>1.001</v>
       </c>
       <c r="G102" t="n">
-        <v>2.904</v>
+        <v>2.595</v>
       </c>
       <c r="H102" t="n">
         <v>260.96</v>
@@ -7756,22 +7756,22 @@
         <v>2002</v>
       </c>
       <c r="B103" t="n">
-        <v>0.647</v>
+        <v>0.548</v>
       </c>
       <c r="C103" t="n">
-        <v>1.733</v>
+        <v>1.469</v>
       </c>
       <c r="D103" t="n">
-        <v>0.236</v>
+        <v>0.2</v>
       </c>
       <c r="E103" t="n">
-        <v>0.632</v>
+        <v>0.535</v>
       </c>
       <c r="F103" t="n">
-        <v>10.568</v>
+        <v>9.151</v>
       </c>
       <c r="G103" t="n">
-        <v>27.393</v>
+        <v>23.719</v>
       </c>
       <c r="H103" t="n">
         <v>119.9</v>
@@ -7849,22 +7849,22 @@
         <v>2003</v>
       </c>
       <c r="B104" t="n">
-        <v>0.772</v>
+        <v>0.646</v>
       </c>
       <c r="C104" t="n">
-        <v>2.068</v>
+        <v>1.731</v>
       </c>
       <c r="D104" t="n">
-        <v>0.225</v>
+        <v>0.184</v>
       </c>
       <c r="E104" t="n">
-        <v>0.602</v>
+        <v>0.492</v>
       </c>
       <c r="F104" t="n">
-        <v>24.864</v>
+        <v>19.985</v>
       </c>
       <c r="G104" t="n">
-        <v>64.447</v>
+        <v>51.801</v>
       </c>
       <c r="H104" t="n">
         <v>188.57</v>
@@ -7930,22 +7930,22 @@
         <v>2004</v>
       </c>
       <c r="B105" t="n">
-        <v>0.975</v>
+        <v>0.762</v>
       </c>
       <c r="C105" t="n">
-        <v>2.61</v>
+        <v>2.041</v>
       </c>
       <c r="D105" t="n">
-        <v>0.224</v>
+        <v>0.175</v>
       </c>
       <c r="E105" t="n">
-        <v>0.6</v>
+        <v>0.469</v>
       </c>
       <c r="F105" t="n">
-        <v>3.261</v>
+        <v>2.778</v>
       </c>
       <c r="G105" t="n">
-        <v>8.452</v>
+        <v>7.2</v>
       </c>
       <c r="H105" t="n">
         <v>107.78</v>
@@ -8039,22 +8039,22 @@
         <v>2005</v>
       </c>
       <c r="B106" t="n">
-        <v>0.608</v>
+        <v>0.542</v>
       </c>
       <c r="C106" t="n">
-        <v>1.63</v>
+        <v>1.452</v>
       </c>
       <c r="D106" t="n">
-        <v>0.149</v>
+        <v>0.13</v>
       </c>
       <c r="E106" t="n">
-        <v>0.4</v>
+        <v>0.347</v>
       </c>
       <c r="F106" t="n">
-        <v>3.913</v>
+        <v>3.513</v>
       </c>
       <c r="G106" t="n">
-        <v>10.142</v>
+        <v>9.105</v>
       </c>
       <c r="H106" t="n">
         <v>46.02</v>
@@ -8148,22 +8148,22 @@
         <v>2006</v>
       </c>
       <c r="B107" t="n">
-        <v>0.779</v>
+        <v>0.675</v>
       </c>
       <c r="C107" t="n">
-        <v>2.087</v>
+        <v>1.807</v>
       </c>
       <c r="D107" t="n">
-        <v>0.192</v>
+        <v>0.162</v>
       </c>
       <c r="E107" t="n">
-        <v>0.513</v>
+        <v>0.433</v>
       </c>
       <c r="F107" t="n">
-        <v>3.4</v>
+        <v>2.819</v>
       </c>
       <c r="G107" t="n">
-        <v>8.814</v>
+        <v>7.308</v>
       </c>
       <c r="H107" t="n">
         <v>88.15000000000001</v>
@@ -8257,22 +8257,22 @@
         <v>2007</v>
       </c>
       <c r="B108" t="n">
-        <v>0.312</v>
+        <v>0.281</v>
       </c>
       <c r="C108" t="n">
-        <v>0.836</v>
+        <v>0.753</v>
       </c>
       <c r="D108" t="n">
-        <v>0.144</v>
+        <v>0.128</v>
       </c>
       <c r="E108" t="n">
-        <v>0.386</v>
+        <v>0.344</v>
       </c>
       <c r="F108" t="n">
-        <v>3.039</v>
+        <v>2.775</v>
       </c>
       <c r="G108" t="n">
-        <v>7.878</v>
+        <v>7.194</v>
       </c>
       <c r="H108" t="n">
         <v>194.8</v>
@@ -8366,22 +8366,22 @@
         <v>2008</v>
       </c>
       <c r="B109" t="n">
-        <v>0.533</v>
+        <v>0.473</v>
       </c>
       <c r="C109" t="n">
-        <v>1.427</v>
+        <v>1.267</v>
       </c>
       <c r="D109" t="n">
-        <v>0.183</v>
+        <v>0.159</v>
       </c>
       <c r="E109" t="n">
-        <v>0.489</v>
+        <v>0.426</v>
       </c>
       <c r="F109" t="n">
-        <v>8.925000000000001</v>
+        <v>7.403</v>
       </c>
       <c r="G109" t="n">
-        <v>23.134</v>
+        <v>19.188</v>
       </c>
       <c r="H109" t="n">
         <v>243.99</v>
@@ -8475,22 +8475,22 @@
         <v>2009</v>
       </c>
       <c r="B110" t="n">
-        <v>0.9419999999999999</v>
+        <v>0.76</v>
       </c>
       <c r="C110" t="n">
-        <v>2.523</v>
+        <v>2.036</v>
       </c>
       <c r="D110" t="n">
-        <v>0.232</v>
+        <v>0.184</v>
       </c>
       <c r="E110" t="n">
-        <v>0.622</v>
+        <v>0.493</v>
       </c>
       <c r="F110" t="n">
-        <v>4.716</v>
+        <v>3.815</v>
       </c>
       <c r="G110" t="n">
-        <v>12.223</v>
+        <v>9.888</v>
       </c>
       <c r="H110" t="n">
         <v>56.37</v>
@@ -8584,22 +8584,22 @@
         <v>2010</v>
       </c>
       <c r="B111" t="n">
-        <v>0.516</v>
+        <v>0.457</v>
       </c>
       <c r="C111" t="n">
-        <v>1.382</v>
+        <v>1.225</v>
       </c>
       <c r="D111" t="n">
-        <v>0.158</v>
+        <v>0.137</v>
       </c>
       <c r="E111" t="n">
-        <v>0.422</v>
+        <v>0.366</v>
       </c>
       <c r="F111" t="n">
-        <v>28.504</v>
+        <v>23.616</v>
       </c>
       <c r="G111" t="n">
-        <v>73.88200000000001</v>
+        <v>61.213</v>
       </c>
       <c r="H111" t="n">
         <v>40.14</v>
@@ -8693,22 +8693,22 @@
         <v>2011</v>
       </c>
       <c r="B112" t="n">
-        <v>0.9320000000000001</v>
+        <v>0.742</v>
       </c>
       <c r="C112" t="n">
-        <v>2.497</v>
+        <v>1.986</v>
       </c>
       <c r="D112" t="n">
-        <v>0.222</v>
+        <v>0.173</v>
       </c>
       <c r="E112" t="n">
-        <v>0.594</v>
+        <v>0.463</v>
       </c>
       <c r="F112" t="n">
-        <v>6.568</v>
+        <v>5.305</v>
       </c>
       <c r="G112" t="n">
-        <v>17.023</v>
+        <v>13.751</v>
       </c>
       <c r="H112" t="n">
         <v>169.64</v>
@@ -8802,22 +8802,22 @@
         <v>2012</v>
       </c>
       <c r="B113" t="n">
-        <v>0.729</v>
+        <v>0.593</v>
       </c>
       <c r="C113" t="n">
-        <v>1.953</v>
+        <v>1.589</v>
       </c>
       <c r="D113" t="n">
-        <v>0.152</v>
+        <v>0.122</v>
       </c>
       <c r="E113" t="n">
-        <v>0.407</v>
+        <v>0.327</v>
       </c>
       <c r="F113" t="n">
-        <v>4.963</v>
+        <v>4.254</v>
       </c>
       <c r="G113" t="n">
-        <v>12.863</v>
+        <v>11.027</v>
       </c>
       <c r="H113" t="n">
         <v>22.41</v>
@@ -8911,22 +8911,22 @@
         <v>2013</v>
       </c>
       <c r="B114" t="n">
-        <v>0.919</v>
+        <v>0.737</v>
       </c>
       <c r="C114" t="n">
-        <v>2.462</v>
+        <v>1.974</v>
       </c>
       <c r="D114" t="n">
-        <v>0.261</v>
+        <v>0.206</v>
       </c>
       <c r="E114" t="n">
-        <v>0.699</v>
+        <v>0.551</v>
       </c>
       <c r="F114" t="n">
-        <v>7.791</v>
+        <v>6.366</v>
       </c>
       <c r="G114" t="n">
-        <v>20.195</v>
+        <v>16.502</v>
       </c>
       <c r="H114" t="n">
         <v>515.25</v>
@@ -9020,22 +9020,22 @@
         <v>2014</v>
       </c>
       <c r="B115" t="n">
-        <v>1.022</v>
+        <v>0.785</v>
       </c>
       <c r="C115" t="n">
-        <v>2.736</v>
+        <v>2.102</v>
       </c>
       <c r="D115" t="n">
-        <v>0.223</v>
+        <v>0.175</v>
       </c>
       <c r="E115" t="n">
-        <v>0.598</v>
+        <v>0.469</v>
       </c>
       <c r="F115" t="n">
-        <v>0.583</v>
+        <v>0.511</v>
       </c>
       <c r="G115" t="n">
-        <v>1.51</v>
+        <v>1.325</v>
       </c>
       <c r="H115" t="n">
         <v>53.3</v>
@@ -9129,22 +9129,22 @@
         <v>2015</v>
       </c>
       <c r="B116" t="n">
-        <v>0.552</v>
+        <v>0.471</v>
       </c>
       <c r="C116" t="n">
-        <v>1.478</v>
+        <v>1.262</v>
       </c>
       <c r="D116" t="n">
-        <v>0.247</v>
+        <v>0.213</v>
       </c>
       <c r="E116" t="n">
-        <v>0.662</v>
+        <v>0.571</v>
       </c>
       <c r="F116" t="n">
-        <v>2.992</v>
+        <v>2.605</v>
       </c>
       <c r="G116" t="n">
-        <v>7.755</v>
+        <v>6.753</v>
       </c>
       <c r="H116" t="n">
         <v>197.44</v>
@@ -9238,22 +9238,22 @@
         <v>2016</v>
       </c>
       <c r="B117" t="n">
-        <v>0.543</v>
+        <v>0.447</v>
       </c>
       <c r="C117" t="n">
-        <v>1.455</v>
+        <v>1.198</v>
       </c>
       <c r="D117" t="n">
-        <v>0.172</v>
+        <v>0.135</v>
       </c>
       <c r="E117" t="n">
-        <v>0.461</v>
+        <v>0.363</v>
       </c>
       <c r="F117" t="n">
-        <v>4.208</v>
+        <v>3.423</v>
       </c>
       <c r="G117" t="n">
-        <v>10.908</v>
+        <v>8.872</v>
       </c>
       <c r="H117" t="n">
         <v>140.42</v>
@@ -9347,22 +9347,22 @@
         <v>2017</v>
       </c>
       <c r="B118" t="n">
-        <v>0.75</v>
+        <v>0.593</v>
       </c>
       <c r="C118" t="n">
-        <v>2.009</v>
+        <v>1.587</v>
       </c>
       <c r="D118" t="n">
-        <v>0.205</v>
+        <v>0.164</v>
       </c>
       <c r="E118" t="n">
-        <v>0.55</v>
+        <v>0.438</v>
       </c>
       <c r="F118" t="n">
-        <v>8.567</v>
+        <v>7.434</v>
       </c>
       <c r="G118" t="n">
-        <v>22.206</v>
+        <v>19.268</v>
       </c>
       <c r="H118" t="n">
         <v>84.90000000000001</v>
@@ -9456,22 +9456,22 @@
         <v>2018</v>
       </c>
       <c r="B119" t="n">
-        <v>0.965</v>
+        <v>0.793</v>
       </c>
       <c r="C119" t="n">
-        <v>2.584</v>
+        <v>2.123</v>
       </c>
       <c r="D119" t="n">
-        <v>0.246</v>
+        <v>0.198</v>
       </c>
       <c r="E119" t="n">
-        <v>0.66</v>
+        <v>0.531</v>
       </c>
       <c r="F119" t="n">
-        <v>10.822</v>
+        <v>9.228999999999999</v>
       </c>
       <c r="G119" t="n">
-        <v>28.051</v>
+        <v>23.921</v>
       </c>
       <c r="H119" t="n">
         <v>102.21</v>
@@ -9565,22 +9565,22 @@
         <v>2019</v>
       </c>
       <c r="B120" t="n">
-        <v>0.741</v>
+        <v>0.585</v>
       </c>
       <c r="C120" t="n">
-        <v>1.985</v>
+        <v>1.566</v>
       </c>
       <c r="D120" t="n">
-        <v>0.205</v>
+        <v>0.161</v>
       </c>
       <c r="E120" t="n">
-        <v>0.55</v>
+        <v>0.432</v>
       </c>
       <c r="F120" t="n">
-        <v>3.062</v>
+        <v>2.554</v>
       </c>
       <c r="G120" t="n">
-        <v>7.937</v>
+        <v>6.621</v>
       </c>
       <c r="H120" t="n">
         <v>144.35</v>
@@ -9674,22 +9674,22 @@
         <v>2020</v>
       </c>
       <c r="B121" t="n">
-        <v>1.003</v>
+        <v>0.8149999999999999</v>
       </c>
       <c r="C121" t="n">
-        <v>2.686</v>
+        <v>2.182</v>
       </c>
       <c r="D121" t="n">
-        <v>0.439</v>
+        <v>0.361</v>
       </c>
       <c r="E121" t="n">
-        <v>1.176</v>
+        <v>0.966</v>
       </c>
       <c r="F121" t="n">
-        <v>1.327</v>
+        <v>1.151</v>
       </c>
       <c r="G121" t="n">
-        <v>3.439</v>
+        <v>2.983</v>
       </c>
       <c r="H121" t="n">
         <v>211.06</v>
@@ -9787,22 +9787,22 @@
         <v>2021</v>
       </c>
       <c r="B122" t="n">
-        <v>0.495</v>
+        <v>0.418</v>
       </c>
       <c r="C122" t="n">
-        <v>1.327</v>
+        <v>1.121</v>
       </c>
       <c r="D122" t="n">
-        <v>0.859</v>
+        <v>0.758</v>
       </c>
       <c r="E122" t="n">
-        <v>2.301</v>
+        <v>2.03</v>
       </c>
       <c r="F122" t="n">
-        <v>2.895</v>
+        <v>2.239</v>
       </c>
       <c r="G122" t="n">
-        <v>7.504</v>
+        <v>5.803</v>
       </c>
       <c r="H122" t="n">
         <v>222.52</v>
@@ -9900,22 +9900,22 @@
         <v>2022</v>
       </c>
       <c r="B123" t="n">
-        <v>1.51</v>
+        <v>1.224</v>
       </c>
       <c r="C123" t="n">
-        <v>4.044</v>
+        <v>3.279</v>
       </c>
       <c r="D123" t="n">
-        <v>0.503</v>
+        <v>0.403</v>
       </c>
       <c r="E123" t="n">
-        <v>1.348</v>
+        <v>1.08</v>
       </c>
       <c r="F123" t="n">
-        <v>6.268</v>
+        <v>5.503</v>
       </c>
       <c r="G123" t="n">
-        <v>16.248</v>
+        <v>14.263</v>
       </c>
       <c r="H123" t="n">
         <v>100.34</v>
@@ -10009,22 +10009,22 @@
         <v>2023</v>
       </c>
       <c r="B124" t="n">
-        <v>1.244</v>
+        <v>1.058</v>
       </c>
       <c r="C124" t="n">
-        <v>3.331</v>
+        <v>2.835</v>
       </c>
       <c r="D124" t="n">
-        <v>0.426</v>
+        <v>0.344</v>
       </c>
       <c r="E124" t="n">
-        <v>1.142</v>
+        <v>0.921</v>
       </c>
       <c r="F124" t="n">
-        <v>4.527</v>
+        <v>3.643</v>
       </c>
       <c r="G124" t="n">
-        <v>11.734</v>
+        <v>9.444000000000001</v>
       </c>
       <c r="H124" t="n">
         <v>71.11</v>
@@ -10118,22 +10118,22 @@
         <v>2024</v>
       </c>
       <c r="B125" t="n">
-        <v>0.859</v>
+        <v>0.678</v>
       </c>
       <c r="C125" t="n">
-        <v>2.3</v>
+        <v>1.815</v>
       </c>
       <c r="D125" t="n">
-        <v>0.274</v>
+        <v>0.219</v>
       </c>
       <c r="E125" t="n">
-        <v>0.734</v>
+        <v>0.588</v>
       </c>
       <c r="F125" t="n">
-        <v>14.916</v>
+        <v>12.022</v>
       </c>
       <c r="G125" t="n">
-        <v>38.663</v>
+        <v>31.16</v>
       </c>
       <c r="H125" t="n">
         <v>91.19</v>
@@ -10227,22 +10227,22 @@
         <v>2025</v>
       </c>
       <c r="B126" t="n">
-        <v>1.014</v>
+        <v>0.784</v>
       </c>
       <c r="C126" t="n">
-        <v>2.715</v>
+        <v>2.099</v>
       </c>
       <c r="D126" t="n">
-        <v>0.312</v>
+        <v>0.243</v>
       </c>
       <c r="E126" t="n">
-        <v>0.835</v>
+        <v>0.65</v>
       </c>
       <c r="F126" t="n">
-        <v>14.157</v>
+        <v>11.563</v>
       </c>
       <c r="G126" t="n">
-        <v>36.696</v>
+        <v>29.97</v>
       </c>
       <c r="H126" t="n">
         <v>187.54</v>
@@ -10336,22 +10336,22 @@
         <v>2026</v>
       </c>
       <c r="B127" t="n">
-        <v>0.962</v>
+        <v>0.755</v>
       </c>
       <c r="C127" t="n">
-        <v>2.577</v>
+        <v>2.022</v>
       </c>
       <c r="D127" t="n">
-        <v>0.3</v>
+        <v>0.229</v>
       </c>
       <c r="E127" t="n">
-        <v>0.804</v>
+        <v>0.614</v>
       </c>
       <c r="F127" t="n">
-        <v>21.627</v>
+        <v>16.823</v>
       </c>
       <c r="G127" t="n">
-        <v>56.056</v>
+        <v>43.604</v>
       </c>
       <c r="H127" t="inlineStr"/>
       <c r="I127" t="inlineStr"/>
@@ -10472,7 +10472,7 @@
       </c>
       <c r="B3" t="inlineStr">
         <is>
-          <t>GEOGLOWS v2 modelled daily flow, river segment 441006241: the Nakatiya at Saidpur Khajuria (28.338 N, 79.471 E), river km 33-34 from the mapped head, just before the city. MODELLED, NOT MEASURED: ERA5 rain-runoff routed down the river network; it knows nothing of the city, canals, pumping, sewage or seepage, and runs 1.6-1.9 times above the real Ramganga at Chaubari. Use it for year-to-year climate swings, not as the river's real volume. 1940-41 are real ERA5 drought years.</t>
+          <t>GEOGLOWS v2 modelled daily flow, river segment 441105311: the Nakatiya at Khajuriya ghat by the Pilibhit bypass (28.3621 N, 79.4754 E), river km 29.4 from the mapped head, just before the city; the segment runs km 27-29 and its catchment is about 148 km2 (estimated). MODELLED, NOT MEASURED: ERA5 rain-runoff routed down the river network; it knows nothing of the city, canals, pumping, sewage or seepage, and runs 1.6-1.9 times above the real Ramganga at Chaubari. Use it for year-to-year climate swings, not as the river's real volume. 1940-41 are real ERA5 drought years.</t>
         </is>
       </c>
     </row>
@@ -10491,12 +10491,12 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>Is 'Khajuriya ghat' right?</t>
+          <t>Where is Khajuriya ghat?</t>
         </is>
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>OpenStreetMap has Saidpur Khajuria 220 m from the channel on the city's northern side; no place named Khajuriya ghat was found in maps. Please confirm the spot; any other point on the river can be swapped in.</t>
+          <t>Located by the user near the Pilibhit bypass road (Suncity Vistar), 186 m from the mapped channel at river km 29.4. Saidpur Khajuria, about 4.6 km downstream (km 34), is a different place.</t>
         </is>
       </c>
     </row>
@@ -10544,7 +10544,7 @@
       </c>
       <c r="B9" t="inlineStr">
         <is>
-          <t>data/nakatiya_watershed.geojson: MERIT-Hydro 90 m delineation (Global Watersheds API). Whole river 444 km2; to Khajuria 235 km2. On flat plains the line is good to a few hundred metres; roads, canals and drains move water across it.</t>
+          <t>data/nakatiya_watershed.geojson: MERIT-Hydro 90 m delineation (Global Watersheds API). Whole river 444 km2; to Khajuriya ghat 200 km2. On flat plains the line is good to a few hundred metres; roads, canals and drains move water across it.</t>
         </is>
       </c>
     </row>

</xml_diff>